<commit_message>
feat(security): SEC-12~15 — R-SEC22(a)/R-SEC24/R-SEC25, six-workbook delivery (124 TC, 70/70), EXEC_GUIDE with environment knowledge
</commit_message>
<xml_diff>
--- a/features/security/sandbox/batch3/security_batch3_v01.xlsx
+++ b/features/security/sandbox/batch3/security_batch3_v01.xlsx
@@ -10494,7 +10494,8 @@
           <t xml:space="preserve">verification: document review (R-SEC23; upstream DR-a/i/r pending)
 source: 037 SWE1-LOGENC-004 Requirement Description and Verification Criteria
 sibling axis: symmetric algorithm; rule R-SEC23(b) VC THEN 3.1
-channel_feasible: N/N</t>
+channel_feasible: N/N
+conflict: 376/509/511 vs 510 vs 514 — key strength; unresolved per CCVR Mapping notes row 14</t>
         </is>
       </c>
     </row>
@@ -10631,7 +10632,8 @@
           <t xml:space="preserve">verification: document review (R-SEC23; upstream DR-a/i/r pending)
 source: 037 SWE1-LOGENC-004 Requirement Description and Verification Criteria
 sibling axis: key generation source; rule R-SEC23(b) VC trailing sentence (independent requirement outside THEN)
-channel_feasible: N/N</t>
+channel_feasible: N/N
+conflict: 376/509/511 vs 510 vs 514 — key strength; unresolved per CCVR Mapping notes row 14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(security): SEC-12 — R-SEC22(a) amend, A-SEC-11~14, ACCEPTED_GAP, security_v07
</commit_message>
<xml_diff>
--- a/features/security/sandbox/batch3/security_batch3_v01.xlsx
+++ b/features/security/sandbox/batch3/security_batch3_v01.xlsx
@@ -10494,7 +10494,8 @@
           <t xml:space="preserve">verification: document review (R-SEC23; upstream DR-a/i/r pending)
 source: 037 SWE1-LOGENC-004 Requirement Description and Verification Criteria
 sibling axis: symmetric algorithm; rule R-SEC23(b) VC THEN 3.1
-channel_feasible: N/N</t>
+channel_feasible: N/N
+conflict: 376/509/511 vs 510 vs 514 — key strength; unresolved per CCVR Mapping notes row 14</t>
         </is>
       </c>
     </row>
@@ -10631,7 +10632,8 @@
           <t xml:space="preserve">verification: document review (R-SEC23; upstream DR-a/i/r pending)
 source: 037 SWE1-LOGENC-004 Requirement Description and Verification Criteria
 sibling axis: key generation source; rule R-SEC23(b) VC trailing sentence (independent requirement outside THEN)
-channel_feasible: N/N</t>
+channel_feasible: N/N
+conflict: 376/509/511 vs 510 vs 514 — key strength; unresolved per CCVR Mapping notes row 14</t>
         </is>
       </c>
     </row>

</xml_diff>